<commit_message>
fix: generate sheet XMLs before shared strings (was empty, now 249 strings)
</commit_message>
<xml_diff>
--- a/docs/design-docs/01_システム概要書.xlsx
+++ b/docs/design-docs/01_システム概要書.xlsx
@@ -10,7 +10,755 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
+  <si>
+    <t>版数</t>
+  </si>
+  <si>
+    <t>改訂日</t>
+  </si>
+  <si>
+    <t>改訂内容</t>
+  </si>
+  <si>
+    <t>改訂者</t>
+  </si>
+  <si>
+    <t>承認者</t>
+  </si>
+  <si>
+    <t>区分</t>
+  </si>
+  <si>
+    <t>備考</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>2026/05/23</t>
+  </si>
+  <si>
+    <t>初版作成</t>
+  </si>
+  <si>
+    <t>システム開発部</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>新規</t>
+  </si>
+  <si>
+    <t>システム概要書</t>
+  </si>
+  <si>
+    <t>文書管理情報</t>
+  </si>
+  <si>
+    <t>システムID</t>
+  </si>
+  <si>
+    <t>STRUTSLAB-001</t>
+  </si>
+  <si>
+    <t>システム名</t>
+  </si>
+  <si>
+    <t>電力設備巡視点検管理システム</t>
+  </si>
+  <si>
+    <t>サブシステム名</t>
+  </si>
+  <si>
+    <t>開発言語</t>
+  </si>
+  <si>
+    <t>Java 1.8 / Struts1 / MyBatis</t>
+  </si>
+  <si>
+    <t>データベース</t>
+  </si>
+  <si>
+    <t>H2 Database（ファイルモード）</t>
+  </si>
+  <si>
+    <t>文書番号</t>
+  </si>
+  <si>
+    <t>作成日</t>
+  </si>
+  <si>
+    <t>作成者</t>
+  </si>
+  <si>
+    <t>システムアーキテクチャ</t>
+  </si>
+  <si>
+    <t>レイヤー</t>
+  </si>
+  <si>
+    <t>採用技術</t>
+  </si>
+  <si>
+    <t>バージョン</t>
+  </si>
+  <si>
+    <t>役割</t>
+  </si>
+  <si>
+    <t>プレゼンテーション層</t>
+  </si>
+  <si>
+    <t>Struts 1.3</t>
+  </si>
+  <si>
+    <t>1.3.10</t>
+  </si>
+  <si>
+    <t>ActionServlet, Action, ActionForm, JSP</t>
+  </si>
+  <si>
+    <t>Tiles</t>
+  </si>
+  <si>
+    <t>画面レイアウト共通化（header/body/footer/menu）</t>
+  </si>
+  <si>
+    <t>JSP + カスタムタグ</t>
+  </si>
+  <si>
+    <t>スクリプトレット主体、独自タグライブラリ</t>
+  </si>
+  <si>
+    <t>ビジネスロジック層</t>
+  </si>
+  <si>
+    <t>Actionクラス</t>
+  </si>
+  <si>
+    <t>Struts1 Action + DispatchAction</t>
+  </si>
+  <si>
+    <t>データアクセス層</t>
+  </si>
+  <si>
+    <t>MyBatis</t>
+  </si>
+  <si>
+    <t>3.5.x</t>
+  </si>
+  <si>
+    <t>SQLマッピング、Mapper.xml</t>
+  </si>
+  <si>
+    <t>H2 Database</t>
+  </si>
+  <si>
+    <t>1.4.200</t>
+  </si>
+  <si>
+    <t>ファイルモード（~/struts-lab-db）</t>
+  </si>
+  <si>
+    <t>バリデーション</t>
+  </si>
+  <si>
+    <t>Validator Plug-in</t>
+  </si>
+  <si>
+    <t>validation.xml, validation-rules.xml</t>
+  </si>
+  <si>
+    <t>ビルドツール</t>
+  </si>
+  <si>
+    <t>Maven</t>
+  </si>
+  <si>
+    <t>3.x</t>
+  </si>
+  <si>
+    <t>war → Tomcat 8.x にデプロイ</t>
+  </si>
+  <si>
+    <t>サーブレットコンテナ</t>
+  </si>
+  <si>
+    <t>Apache Tomcat</t>
+  </si>
+  <si>
+    <t>8.5.x</t>
+  </si>
+  <si>
+    <t>Java 1.8 対応</t>
+  </si>
+  <si>
+    <t>機能モジュール一覧</t>
+  </si>
+  <si>
+    <t>モジュール名</t>
+  </si>
+  <si>
+    <t>略称</t>
+  </si>
+  <si>
+    <t>対象画面数</t>
+  </si>
+  <si>
+    <t>主なテスト難点</t>
+  </si>
+  <si>
+    <t>マスタ管理</t>
+  </si>
+  <si>
+    <t>MASTER</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>多段検索、ツリー選択、親子設定、CSV出力</t>
+  </si>
+  <si>
+    <t>点検計画・実施</t>
+  </si>
+  <si>
+    <t>INSPECT</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Wizard、ネストチェック、写真添付、条件付きバリデーション、承認フロー</t>
+  </si>
+  <si>
+    <t>異常報告</t>
+  </si>
+  <si>
+    <t>INCIDENT</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>ステータス遷移、条件付き必須項目、類似事例検索</t>
+  </si>
+  <si>
+    <t>対応指示・是正</t>
+  </si>
+  <si>
+    <t>COUNTER</t>
+  </si>
+  <si>
+    <t>動的行追加、Nested Properties、ポップアップ選択、全明細完了チェック</t>
+  </si>
+  <si>
+    <t>組織・要員管理</t>
+  </si>
+  <si>
+    <t>ORG</t>
+  </si>
+  <si>
+    <t>階層ツリー、資格期限チェック、多セクションフォーム</t>
+  </si>
+  <si>
+    <t>カレンダー・休日</t>
+  </si>
+  <si>
+    <t>CALENDAR</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>カレンダー表示、一括登録、重複チェック</t>
+  </si>
+  <si>
+    <t>保守部品管理</t>
+  </si>
+  <si>
+    <t>PARTS</t>
+  </si>
+  <si>
+    <t>チェックボックスツリー、在庫アラート、数量自動引当</t>
+  </si>
+  <si>
+    <t>レポート</t>
+  </si>
+  <si>
+    <t>REPORT</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>クロス集計、テーブル形式グラフ、期間指定</t>
+  </si>
+  <si>
+    <t>画面一覧（全27画面）</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>モジュール</t>
+  </si>
+  <si>
+    <t>画面ID</t>
+  </si>
+  <si>
+    <t>画面名</t>
+  </si>
+  <si>
+    <t>種別</t>
+  </si>
+  <si>
+    <t>主要Struts1要素</t>
+  </si>
+  <si>
+    <t>テスト難点</t>
+  </si>
+  <si>
+    <t>SCR-MST-EQP-001</t>
+  </si>
+  <si>
+    <t>設備マスタ一覧</t>
+  </si>
+  <si>
+    <t>一覧</t>
+  </si>
+  <si>
+    <t>Action,Form,Paging</t>
+  </si>
+  <si>
+    <t>多段検索,一括操作,CSV</t>
+  </si>
+  <si>
+    <t>SCR-MST-EQP-002</t>
+  </si>
+  <si>
+    <t>設備マスタ登録・編集</t>
+  </si>
+  <si>
+    <t>登録</t>
+  </si>
+  <si>
+    <t>Form,Validator,Popup</t>
+  </si>
+  <si>
+    <t>条件付き必須,Popup→親画面</t>
+  </si>
+  <si>
+    <t>SCR-MST-CHK-001</t>
+  </si>
+  <si>
+    <t>点検項目マスタ一覧</t>
+  </si>
+  <si>
+    <t>Action,Form</t>
+  </si>
+  <si>
+    <t>テンプレートコピー,並順変更</t>
+  </si>
+  <si>
+    <t>SCR-MST-CHK-002</t>
+  </si>
+  <si>
+    <t>点検項目マスタ登録編集</t>
+  </si>
+  <si>
+    <t>DispatchAction,動的行</t>
+  </si>
+  <si>
+    <t>3階層ツリー編集</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>SCR-INS-PLAN-001</t>
+  </si>
+  <si>
+    <t>年間点検計画一覧</t>
+  </si>
+  <si>
+    <t>マトリクス表示(動的カラム)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>SCR-INS-PLAN-002</t>
+  </si>
+  <si>
+    <t>点検計画登録（Wizard）</t>
+  </si>
+  <si>
+    <t>Form,Wizard 4step</t>
+  </si>
+  <si>
+    <t>マルチステップ,途中復帰</t>
+  </si>
+  <si>
+    <t>SCR-INS-DAILY-001</t>
+  </si>
+  <si>
+    <t>点検実施一覧（当日）</t>
+  </si>
+  <si>
+    <t>バッジ,直接遷移</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>SCR-INS-EXEC-001</t>
+  </si>
+  <si>
+    <t>点検実施入力</t>
+  </si>
+  <si>
+    <t>入力</t>
+  </si>
+  <si>
+    <t>Form,FileUpload,Validator</t>
+  </si>
+  <si>
+    <t>ネスト,条件付き,写真</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>SCR-INS-EXEC-002</t>
+  </si>
+  <si>
+    <t>点検実施詳細・修正</t>
+  </si>
+  <si>
+    <t>表示</t>
+  </si>
+  <si>
+    <t>Form,Validator</t>
+  </si>
+  <si>
+    <t>修正申請→承認フロー</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>SCR-INS-APPR-001</t>
+  </si>
+  <si>
+    <t>点検実施承認一覧</t>
+  </si>
+  <si>
+    <t>Action,一括操作</t>
+  </si>
+  <si>
+    <t>一括承認/差戻し</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>SCR-INC-LIST-001</t>
+  </si>
+  <si>
+    <t>異常報告一覧</t>
+  </si>
+  <si>
+    <t>7条件複合検索,条件保存</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>SCR-INC-CREATE-001</t>
+  </si>
+  <si>
+    <t>異常報告登録</t>
+  </si>
+  <si>
+    <t>Form,FileUpload</t>
+  </si>
+  <si>
+    <t>データ引継,類似事例</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>SCR-INC-DETAIL-001</t>
+  </si>
+  <si>
+    <t>異常報告詳細</t>
+  </si>
+  <si>
+    <t>詳細</t>
+  </si>
+  <si>
+    <t>Form,LookupDispatch</t>
+  </si>
+  <si>
+    <t>多段階遷移</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>SCR-CTR-CREATE-001</t>
+  </si>
+  <si>
+    <t>対応指示登録</t>
+  </si>
+  <si>
+    <t>Form,Indexed,Popup</t>
+  </si>
+  <si>
+    <t>動的行(Submit),index再振</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>SCR-CTR-LIST-001</t>
+  </si>
+  <si>
+    <t>対応指示一覧</t>
+  </si>
+  <si>
+    <t>複合検索,印刷用window</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>SCR-CTR-DETAIL-001</t>
+  </si>
+  <si>
+    <t>対応指示詳細・完了</t>
+  </si>
+  <si>
+    <t>明細個別更新,自動完了</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>SCR-CTR-CAPA-001</t>
+  </si>
+  <si>
+    <t>是正処置報告書</t>
+  </si>
+  <si>
+    <t>なぜなぜ分析5段階</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>SCR-RPT-SUMMARY-001</t>
+  </si>
+  <si>
+    <t>総合レポート</t>
+  </si>
+  <si>
+    <t>クロス集計,擬似グラフ</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>SCR-ORG-DEPT-001</t>
+  </si>
+  <si>
+    <t>部署マスタ一覧</t>
+  </si>
+  <si>
+    <t>4階層ツリー表示</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>SCR-ORG-DEPT-002</t>
+  </si>
+  <si>
+    <t>部署マスタ登録・編集</t>
+  </si>
+  <si>
+    <t>ツリーPopup,過去日</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>SCR-ORG-EMP-001</t>
+  </si>
+  <si>
+    <t>担当者マスタ一覧</t>
+  </si>
+  <si>
+    <t>複合検索,資格期限</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>SCR-ORG-EMP-002</t>
+  </si>
+  <si>
+    <t>担当者マスタ登録・編集</t>
+  </si>
+  <si>
+    <t>5section,認定期限</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>SCR-CAL-LIST-001</t>
+  </si>
+  <si>
+    <t>休日カレンダー一覧</t>
+  </si>
+  <si>
+    <t>月別表示,色分け</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>SCR-CAL-REG-001</t>
+  </si>
+  <si>
+    <t>休日登録・編集</t>
+  </si>
+  <si>
+    <t>範囲一括,重複</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>SCR-PRT-LIST-001</t>
+  </si>
+  <si>
+    <t>保守部品一覧</t>
+  </si>
+  <si>
+    <t>在庫アラート</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>SCR-PRT-REG-001</t>
+  </si>
+  <si>
+    <t>保守部品登録・編集</t>
+  </si>
+  <si>
+    <t>Form,Validator,File</t>
+  </si>
+  <si>
+    <t>checkboxツリー</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>SCR-PRT-USAGE-001</t>
+  </si>
+  <si>
+    <t>部品使用実績一覧</t>
+  </si>
+  <si>
+    <t>在庫自動引当</t>
+  </si>
+  <si>
+    <t>Struts1 設定ファイル構成</t>
+  </si>
+  <si>
+    <t>ファイル</t>
+  </si>
+  <si>
+    <t>配置パス</t>
+  </si>
+  <si>
+    <t>web.xml</t>
+  </si>
+  <si>
+    <t>/WEB-INF/web.xml</t>
+  </si>
+  <si>
+    <t>ActionServlet, Tiles, Validator</t>
+  </si>
+  <si>
+    <t>struts-config.xml</t>
+  </si>
+  <si>
+    <t>/WEB-INF/struts-config.xml</t>
+  </si>
+  <si>
+    <t>Action, FormBean, Forward, Plug-in</t>
+  </si>
+  <si>
+    <t>tiles-defs.xml</t>
+  </si>
+  <si>
+    <t>/WEB-INF/tiles-defs.xml</t>
+  </si>
+  <si>
+    <t>Tilesレイアウト定義</t>
+  </si>
+  <si>
+    <t>validation.xml</t>
+  </si>
+  <si>
+    <t>/WEB-INF/validation.xml</t>
+  </si>
+  <si>
+    <t>Validator検証ルール</t>
+  </si>
+  <si>
+    <t>validator-rules.xml</t>
+  </si>
+  <si>
+    <t>/WEB-INF/validator-rules.xml</t>
+  </si>
+  <si>
+    <t>Validator基本ルール</t>
+  </si>
+  <si>
+    <t>mybatis-config.xml</t>
+  </si>
+  <si>
+    <t>クラスパス直下</t>
+  </si>
+  <si>
+    <t>MyBatis, DataSource, Mapper</t>
+  </si>
+  <si>
+    <t>ApplicationResources_ja.properties</t>
+  </si>
+  <si>
+    <t>日本語メッセージリソース</t>
+  </si>
+  <si>
+    <t>*.tld</t>
+  </si>
+  <si>
+    <t>/WEB-INF/tld/</t>
+  </si>
+  <si>
+    <t>カスタムタグ定義</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>